<commit_message>
Post vacante alianzas: contratacion inmediata
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>En Heiiu English Academy abrimos UNA vacante: Ejecutivo(a) de Alianzas Empresariales.</t>
+          <t>En Heiiu English Academy abrimos UNA vacante de CONTRATACIÓN INMEDIATA: Ejecutivo(a) de Alianzas Empresariales.</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Subtítulo: Abre las puertas de las empresas de Bucaramanga al inglés.</t>
+          <t>Subtítulo: Abre las puertas de las empresas de Bucaramanga al inglés. CONTRATACIÓN INMEDIATA.</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>1. PIEZA PRINCIPAL: crear la vacante gratuita en LinkedIn Empleos desde la página de empresa de Heiiu, con el texto del post (título: Ejecutivo(a) de Alianzas Empresariales · ubicación: Bucaramanga · presencial · tiempo completo). Aparece por búsqueda, no depende de seguidores.</t>
+          <t>1. PIEZA PRINCIPAL: crear la vacante gratuita en LinkedIn Empleos desde la página de empresa de Heiiu, con el texto del post (título: Ejecutivo(a) de Alianzas Empresariales — Contratación inmediata · ubicación: Bucaramanga · presencial · tiempo completo). Aparece por búsqueda, no depende de seguidores.</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>· Contrato: laboral, con período de prueba de ley</t>
+          <t>· Contrato: laboral, con período de prueba de ley · CONTRATACIÓN INMEDIATA</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Hola [NOMBRE], vi tu perfil y tu experiencia en [alianzas / venta corporativa] en [EMPRESA]. En Heiiu English Academy, en Bucaramanga, estamos buscando UNA persona para construir nuestro canal de alianzas con empresas, colegios y fundaciones: contrato laboral, ingreso mínimo garantizado de $3.500.000 los tres primeros meses, 10% de lo que pague cada empresa y cartera mensual por cada estudiante de tus alianzas, sin techo.</t>
+          <t>Hola [NOMBRE], vi tu perfil y tu experiencia en [alianzas / venta corporativa] en [EMPRESA]. En Heiiu English Academy, en Bucaramanga, estamos buscando, para contratación inmediata, UNA persona para construir nuestro canal de alianzas con empresas, colegios y fundaciones: contrato laboral, ingreso mínimo garantizado de $3.500.000 los tres primeros meses, 10% de lo que pague cada empresa y cartera mensual por cada estudiante de tus alianzas, sin techo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pieza grafica vacante alianzas (1080x1350) y correo citasheiiu@gmail.com
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
@@ -569,7 +569,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Envía tu hoja de vida a auxiliaradministrativo@heiiu.com con el asunto "Alianzas Heiiu" y, esto es lo importante, un audio o video de 1 minuto contándonos la alianza o el convenio más importante que hayas cerrado y cómo lo lograste. Sin el audio no revisamos la hoja de vida. En la entrevista nos presentarás la alianza como si fuéramos el gerente de una empresa de 40 empleados.</t>
+          <t>Envía tu hoja de vida a citasheiiu@gmail.com con el asunto "Alianzas Heiiu" y, esto es lo importante, un audio o video de 1 minuto contándonos la alianza o el convenio más importante que hayas cerrado y cómo lo lograste. Sin el audio no revisamos la hoja de vida. En la entrevista nos presentarás la alianza como si fuéramos el gerente de una empresa de 40 empleados.</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>5. Las hojas de vida llegan a auxiliaradministrativo@heiiu.com con el asunto "Alianzas Heiiu".</t>
+          <t>5. Las hojas de vida llegan a citasheiiu@gmail.com con el asunto "Alianzas Heiiu".</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>· Contacto: auxiliaradministrativo@heiiu.com, asunto "Alianzas Heiiu".</t>
+          <t>· Contacto: citasheiiu@gmail.com, asunto "Alianzas Heiiu".</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Correo de recepción: confirmar que auxiliaradministrativo@heiiu.com está activo y que alguien lo revisa a diario; si no, cambiar por el que se use.</t>
+          <t>Correo de recepción: citasheiiu@gmail.com, asunto "Alianzas Heiiu" (filtrar en Gmail por el asunto).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vacante alianzas: Senior, minimo 5 anos, pieza con cifras
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>En Heiiu English Academy abrimos UNA vacante de CONTRATACIÓN INMEDIATA: Ejecutivo(a) de Alianzas Empresariales.</t>
+          <t>En Heiiu English Academy abrimos UNA vacante de CONTRATACIÓN INMEDIATA: Ejecutivo(a) Senior de Alianzas Empresariales.</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>• Experiencia en alianzas estratégicas, convenios o venta corporativa (B2B), idealmente en educación, salud, seguros o servicios.</t>
+          <t>• Mínimo 5 años de experiencia en alianzas estratégicas, convenios o venta corporativa (B2B), idealmente en educación, salud, seguros o servicios.</t>
         </is>
       </c>
     </row>
@@ -614,14 +614,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Titular: BUSCAMOS EJECUTIVO(A) DE ALIANZAS EMPRESARIALES</t>
+          <t>Titular: BUSCAMOS EJECUTIVO(A) SENIOR DE ALIANZAS EMPRESARIALES</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Subtítulo: Abre las puertas de las empresas de Bucaramanga al inglés. CONTRATACIÓN INMEDIATA.</t>
+          <t>Subtítulo: Mínimo 5 años de experiencia B2B. CONTRATACIÓN INMEDIATA.</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>1. PIEZA PRINCIPAL: crear la vacante gratuita en LinkedIn Empleos desde la página de empresa de Heiiu, con el texto del post (título: Ejecutivo(a) de Alianzas Empresariales — Contratación inmediata · ubicación: Bucaramanga · presencial · tiempo completo). Aparece por búsqueda, no depende de seguidores.</t>
+          <t>1. PIEZA PRINCIPAL: crear la vacante gratuita en LinkedIn Empleos desde la página de empresa de Heiiu, con el texto del post (título: Ejecutivo(a) Senior de Alianzas Empresariales — Contratación inmediata · ubicación: Bucaramanga · presencial · tiempo completo). Aparece por búsqueda, no depende de seguidores.</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>· Cargo: Ejecutivo(a) de Alianzas Empresariales</t>
+          <t>· Cargo: Ejecutivo(a) Senior de Alianzas Empresariales</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>· Experiencia: alianzas, convenios o venta corporativa B2B</t>
+          <t>· Experiencia: mínimo 5 años en alianzas, convenios o venta corporativa B2B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Post vacante alianzas regenerado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE_ALIANZAS.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -450,7 +450,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Te lo digo de frente, como le hablamos a nuestros estudiantes: este cargo es de calle y de relaciones con quien decide. Gerentes, talento humano, bienestar, rectores y fundaciones. No atiendes citas que llegan por anuncios: tú construyes el canal corporativo e institucional, y lo haces tuyo.</t>
+          <t>Es un cargo de campo y de relacionamiento con la alta dirección: gerencias, talento humano, bienestar, rectorías y fundaciones. La misión es liderar el canal corporativo e institucional de Heiiu, construirlo y hacerlo crecer, con el respaldo de un equipo comercial y académico.</t>
         </is>
       </c>
     </row>
@@ -520,68 +520,75 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>• Mínimo 5 años de experiencia en alianzas estratégicas, convenios o venta corporativa (B2B), idealmente en educación, salud, seguros o servicios.</t>
+          <t>• Ventas como tu fuerte: mínimo 5 años vendiendo y cerrando negocios corporativos (B2B), alianzas o convenios, con resultados que puedas demostrar con cifras. Idealmente en educación, salud, seguros o servicios.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>• Relacionamiento con gerencias, áreas de talento humano y bienestar; deseable experiencia con colegios, fundaciones o contratación pública.</t>
+          <t>• Cierre con quien decide: gerencias, talento humano, bienestar, rectorías y fundaciones.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>• Ritmo: hablar cada día con quien decide en al menos dos empresas nuevas.</t>
+          <t>• Manejo de números: metas, presupuestos comerciales, indicadores y embudo de ventas. Que leas tu propio tablero y anticipes tus resultados.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>• Disciplina de registro: lo que no está en el tablero, no existe.</t>
+          <t>• Mercadeo y activación: eventos, ferias, charlas corporativas, BTL.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>• Curiosidad para proponer nuevos programas y oportunidades.</t>
+          <t>• Deseable: contratación pública (SECOP), manejo de cartera y recaudo, o liderazgo de equipos comerciales.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>• Trabajo en Bucaramanga y su área metropolitana.</t>
+          <t>• Formación profesional en áreas comerciales, de mercadeo, administración, economía, contaduría o afines.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>• Disciplina de registro, curiosidad para proponer nuevas oportunidades y trabajo en Bucaramanga y su área metropolitana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>CÓMO APLICAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Envía tu hoja de vida a citasheiiu@gmail.com con el asunto "Alianzas Heiiu" y, esto es lo importante, un audio o video de 1 minuto contándonos la alianza o el convenio más importante que hayas cerrado y cómo lo lograste. Sin el audio no revisamos la hoja de vida. En la entrevista nos presentarás la alianza como si fuéramos el gerente de una empresa de 40 empleados.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Si conoces a alguien así, etiquétalo(a). La persona correcta llega a un cargo donde su esfuerzo se nota en su bolsillo.</t>
+          <t>Envía tu hoja de vida a citasheiiu@gmail.com con el asunto "Alianzas Heiiu" y, esto es lo importante, un audio o video de 1 minuto contándonos la alianza o el convenio más importante que hayas cerrado y cómo lo lograste. Sin el audio no revisamos la hoja de vida. En la entrevista nos presentarás la alianza como si fuéramos el gerente de una empresa de 40 empleados.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Si conoces a alguien así, etiquétalo(a). La persona correcta llega a un cargo donde su esfuerzo se nota en su bolsillo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>#Bucaramanga #EmpleoBucaramanga #AlianzasEstratégicas #VentasB2B #DesarrolloDeNegocios #Educación</t>
         </is>
@@ -737,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -802,26 +809,33 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>· Experiencia: mínimo 5 años en alianzas, convenios o venta corporativa B2B</t>
+          <t>· Experiencia: mínimo 5 años en VENTAS corporativas B2B, alianzas o convenios, con resultados demostrables; manejo de indicadores y presupuestos comerciales; mercadeo y activación (deseable SECOP, cartera o liderazgo de equipos)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>· Descripción: copiar el texto de la hoja POST LINKEDIN, sin los hashtags.</t>
+          <t>· Formación: profesional en áreas comerciales, mercadeo, administración, economía, contaduría o afines</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>· Contacto: citasheiiu@gmail.com, asunto "Alianzas Heiiu".</t>
+          <t>· Descripción: copiar el texto de la hoja POST LINKEDIN, sin los hashtags.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>· Contacto: citasheiiu@gmail.com, asunto "Alianzas Heiiu".</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Filtro al recibir: quien no mande el audio o video de 1 minuto queda descartado sin revisar. A los que sí lo manden se les envía la PROPUESTA_EJECUTIVA_ALIANZAS.pdf y se agenda la entrevista con la simulación (presentar la alianza a "un gerente de una empresa de 40 empleados").</t>
         </is>

</xml_diff>